<commit_message>
3/6 : 修正Pearson Panel
</commit_message>
<xml_diff>
--- a/correlation_table_假設1_維度1.xlsx
+++ b/correlation_table_假設1_維度1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,6 +497,11 @@
       <c r="O1" s="1" t="inlineStr">
         <is>
           <t>累計報酬率</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>AI變數</t>
         </is>
       </c>
     </row>
@@ -524,6 +529,7 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -553,6 +559,7 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -586,6 +593,7 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -623,6 +631,7 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -664,6 +673,7 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -709,6 +719,7 @@
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -758,6 +769,7 @@
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -811,6 +823,7 @@
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -868,6 +881,7 @@
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -929,6 +943,7 @@
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -994,6 +1009,7 @@
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -1063,6 +1079,7 @@
       </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
@@ -1136,6 +1153,7 @@
         </is>
       </c>
       <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
@@ -1209,6 +1227,89 @@
         </is>
       </c>
       <c r="O15" t="inlineStr">
+        <is>
+          <t>1.0000</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>AI變數</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0.0298</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>-0.0825***</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0.1313***</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0.0213</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.0282</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>-0.0587**</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>0.1225***</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>0.0798***</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>0.0411*</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>0.0666***</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>-0.2013***</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>0.0265</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>-0.0088</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>0.0631***</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
         <is>
           <t>1.0000</t>
         </is>

</xml_diff>